<commit_message>
update(ai): re run tft_infernece.ipynb
</commit_message>
<xml_diff>
--- a/reports/tft_future_prediction_results.xlsx
+++ b/reports/tft_future_prediction_results.xlsx
@@ -471,19 +471,19 @@
         <v>45839</v>
       </c>
       <c r="B2" t="n">
-        <v>28.06027412414551</v>
+        <v>19.457275390625</v>
       </c>
       <c r="C2" t="n">
-        <v>30.0876407623291</v>
+        <v>26.12072944641113</v>
       </c>
       <c r="D2" t="n">
-        <v>1260.757202148438</v>
+        <v>738.5988159179688</v>
       </c>
       <c r="E2" t="n">
-        <v>29.61800956726074</v>
+        <v>20.0220832824707</v>
       </c>
       <c r="F2" t="n">
-        <v>14.18550968170166</v>
+        <v>15.99444675445557</v>
       </c>
     </row>
     <row r="3">
@@ -491,19 +491,19 @@
         <v>45839.04166666666</v>
       </c>
       <c r="B3" t="n">
-        <v>29.17035675048828</v>
+        <v>19.33887100219727</v>
       </c>
       <c r="C3" t="n">
-        <v>37.20879364013672</v>
+        <v>28.83571434020996</v>
       </c>
       <c r="D3" t="n">
-        <v>1309.504150390625</v>
+        <v>739.6646728515625</v>
       </c>
       <c r="E3" t="n">
-        <v>38.85080718994141</v>
+        <v>25.57710266113281</v>
       </c>
       <c r="F3" t="n">
-        <v>13.71520328521729</v>
+        <v>16.77538871765137</v>
       </c>
     </row>
     <row r="4">
@@ -511,19 +511,19 @@
         <v>45839.08333333334</v>
       </c>
       <c r="B4" t="n">
-        <v>36.28301620483398</v>
+        <v>25.67109870910645</v>
       </c>
       <c r="C4" t="n">
-        <v>48.71586608886719</v>
+        <v>36.02253341674805</v>
       </c>
       <c r="D4" t="n">
-        <v>1931.81494140625</v>
+        <v>1335.839599609375</v>
       </c>
       <c r="E4" t="n">
-        <v>33.05432510375977</v>
+        <v>23.64129066467285</v>
       </c>
       <c r="F4" t="n">
-        <v>20.71739196777344</v>
+        <v>21.70256423950195</v>
       </c>
     </row>
     <row r="5">
@@ -531,19 +531,19 @@
         <v>45839.125</v>
       </c>
       <c r="B5" t="n">
-        <v>28.97974014282227</v>
+        <v>20.21038246154785</v>
       </c>
       <c r="C5" t="n">
-        <v>34.39680862426758</v>
+        <v>25.15389060974121</v>
       </c>
       <c r="D5" t="n">
-        <v>1196.845947265625</v>
+        <v>787.8184814453125</v>
       </c>
       <c r="E5" t="n">
-        <v>35.18789672851562</v>
+        <v>23.35725593566895</v>
       </c>
       <c r="F5" t="n">
-        <v>23.83103370666504</v>
+        <v>24.53015327453613</v>
       </c>
     </row>
     <row r="6">
@@ -551,19 +551,19 @@
         <v>45839.16666666666</v>
       </c>
       <c r="B6" t="n">
-        <v>24.65806198120117</v>
+        <v>17.30211067199707</v>
       </c>
       <c r="C6" t="n">
-        <v>33.08241653442383</v>
+        <v>23.62578392028809</v>
       </c>
       <c r="D6" t="n">
-        <v>683.9907836914062</v>
+        <v>487.873291015625</v>
       </c>
       <c r="E6" t="n">
-        <v>22.77924919128418</v>
+        <v>16.76626777648926</v>
       </c>
       <c r="F6" t="n">
-        <v>19.31797790527344</v>
+        <v>18.37421989440918</v>
       </c>
     </row>
     <row r="7">
@@ -571,19 +571,19 @@
         <v>45839.20833333334</v>
       </c>
       <c r="B7" t="n">
-        <v>19.28565979003906</v>
+        <v>11.72529125213623</v>
       </c>
       <c r="C7" t="n">
-        <v>46.79185485839844</v>
+        <v>38.30211639404297</v>
       </c>
       <c r="D7" t="n">
-        <v>393.48388671875</v>
+        <v>323.4993591308594</v>
       </c>
       <c r="E7" t="n">
-        <v>15.47568511962891</v>
+        <v>13.65237808227539</v>
       </c>
       <c r="F7" t="n">
-        <v>25.80052947998047</v>
+        <v>26.24072265625</v>
       </c>
     </row>
     <row r="8">
@@ -591,19 +591,19 @@
         <v>45839.25</v>
       </c>
       <c r="B8" t="n">
-        <v>22.86503982543945</v>
+        <v>18.11710357666016</v>
       </c>
       <c r="C8" t="n">
-        <v>35.70196914672852</v>
+        <v>29.62737274169922</v>
       </c>
       <c r="D8" t="n">
-        <v>467.2354125976562</v>
+        <v>399.9075317382812</v>
       </c>
       <c r="E8" t="n">
-        <v>13.77951908111572</v>
+        <v>12.13775634765625</v>
       </c>
       <c r="F8" t="n">
-        <v>32.12352752685547</v>
+        <v>35.86870193481445</v>
       </c>
     </row>
     <row r="9">
@@ -611,19 +611,19 @@
         <v>45839.29166666666</v>
       </c>
       <c r="B9" t="n">
-        <v>23.22392272949219</v>
+        <v>17.99732208251953</v>
       </c>
       <c r="C9" t="n">
-        <v>43.59115982055664</v>
+        <v>36.09568405151367</v>
       </c>
       <c r="D9" t="n">
-        <v>446.5171813964844</v>
+        <v>390.1694030761719</v>
       </c>
       <c r="E9" t="n">
-        <v>4.013782024383545</v>
+        <v>6.345967769622803</v>
       </c>
       <c r="F9" t="n">
-        <v>20.30702590942383</v>
+        <v>21.8337230682373</v>
       </c>
     </row>
     <row r="10">
@@ -631,19 +631,19 @@
         <v>45839.33333333334</v>
       </c>
       <c r="B10" t="n">
-        <v>20.64097595214844</v>
+        <v>12.53931713104248</v>
       </c>
       <c r="C10" t="n">
-        <v>33.73042297363281</v>
+        <v>24.55483055114746</v>
       </c>
       <c r="D10" t="n">
-        <v>407.7375183105469</v>
+        <v>373.747802734375</v>
       </c>
       <c r="E10" t="n">
-        <v>9.960555076599121</v>
+        <v>10.33207416534424</v>
       </c>
       <c r="F10" t="n">
-        <v>20.1211986541748</v>
+        <v>21.37019538879395</v>
       </c>
     </row>
     <row r="11">
@@ -651,19 +651,19 @@
         <v>45839.375</v>
       </c>
       <c r="B11" t="n">
-        <v>22.62579536437988</v>
+        <v>16.99173927307129</v>
       </c>
       <c r="C11" t="n">
-        <v>41.09465026855469</v>
+        <v>33.39770126342773</v>
       </c>
       <c r="D11" t="n">
-        <v>429.5667724609375</v>
+        <v>360.5068359375</v>
       </c>
       <c r="E11" t="n">
-        <v>8.40229320526123</v>
+        <v>8.780581474304199</v>
       </c>
       <c r="F11" t="n">
-        <v>27.8209400177002</v>
+        <v>28.01096534729004</v>
       </c>
     </row>
     <row r="12">
@@ -671,19 +671,19 @@
         <v>45839.41666666666</v>
       </c>
       <c r="B12" t="n">
-        <v>32.13529205322266</v>
+        <v>25.42263603210449</v>
       </c>
       <c r="C12" t="n">
-        <v>32.55218887329102</v>
+        <v>23.99739456176758</v>
       </c>
       <c r="D12" t="n">
-        <v>452.2828369140625</v>
+        <v>381.94873046875</v>
       </c>
       <c r="E12" t="n">
-        <v>16.5561466217041</v>
+        <v>13.86325740814209</v>
       </c>
       <c r="F12" t="n">
-        <v>28.02773094177246</v>
+        <v>27.74604225158691</v>
       </c>
     </row>
     <row r="13">
@@ -691,19 +691,19 @@
         <v>45839.45833333334</v>
       </c>
       <c r="B13" t="n">
-        <v>26.44610404968262</v>
+        <v>21.60729217529297</v>
       </c>
       <c r="C13" t="n">
-        <v>36.85089492797852</v>
+        <v>30.55653381347656</v>
       </c>
       <c r="D13" t="n">
-        <v>489.5716552734375</v>
+        <v>393.2742919921875</v>
       </c>
       <c r="E13" t="n">
-        <v>9.43882942199707</v>
+        <v>10.36833190917969</v>
       </c>
       <c r="F13" t="n">
-        <v>16.14228820800781</v>
+        <v>19.06272506713867</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update(ai): re run tft last inference and try without y3
</commit_message>
<xml_diff>
--- a/reports/tft_future_prediction_results.xlsx
+++ b/reports/tft_future_prediction_results.xlsx
@@ -471,19 +471,19 @@
         <v>45839</v>
       </c>
       <c r="B2" t="n">
-        <v>18.74406623840332</v>
+        <v>24.85847473144531</v>
       </c>
       <c r="C2" t="n">
-        <v>25.76019668579102</v>
+        <v>31.48613929748535</v>
       </c>
       <c r="D2" t="n">
-        <v>842.6658325195312</v>
+        <v>851.52197265625</v>
       </c>
       <c r="E2" t="n">
-        <v>19.77779006958008</v>
+        <v>22.50662803649902</v>
       </c>
       <c r="F2" t="n">
-        <v>14.9937572479248</v>
+        <v>14.4581413269043</v>
       </c>
     </row>
     <row r="3">
@@ -491,19 +491,19 @@
         <v>45839.04166666666</v>
       </c>
       <c r="B3" t="n">
-        <v>21.56143569946289</v>
+        <v>28.33466339111328</v>
       </c>
       <c r="C3" t="n">
-        <v>32.96147537231445</v>
+        <v>38.21697998046875</v>
       </c>
       <c r="D3" t="n">
-        <v>969.8318481445312</v>
+        <v>954.2392578125</v>
       </c>
       <c r="E3" t="n">
-        <v>30.42084312438965</v>
+        <v>31.89828300476074</v>
       </c>
       <c r="F3" t="n">
-        <v>14.74695014953613</v>
+        <v>15.23159313201904</v>
       </c>
     </row>
     <row r="4">
@@ -511,19 +511,19 @@
         <v>45839.08333333334</v>
       </c>
       <c r="B4" t="n">
-        <v>29.29644584655762</v>
+        <v>29.22516441345215</v>
       </c>
       <c r="C4" t="n">
-        <v>39.67042922973633</v>
+        <v>37.97681045532227</v>
       </c>
       <c r="D4" t="n">
-        <v>1981.097778320312</v>
+        <v>1635.728149414062</v>
       </c>
       <c r="E4" t="n">
-        <v>27.72442054748535</v>
+        <v>26.40887451171875</v>
       </c>
       <c r="F4" t="n">
-        <v>17.10812759399414</v>
+        <v>19.17269706726074</v>
       </c>
     </row>
     <row r="5">
@@ -531,19 +531,19 @@
         <v>45839.125</v>
       </c>
       <c r="B5" t="n">
-        <v>19.23020172119141</v>
+        <v>21.77865791320801</v>
       </c>
       <c r="C5" t="n">
-        <v>23.00654602050781</v>
+        <v>25.18094635009766</v>
       </c>
       <c r="D5" t="n">
-        <v>1167.433227539062</v>
+        <v>897.946533203125</v>
       </c>
       <c r="E5" t="n">
-        <v>27.33531761169434</v>
+        <v>24.71508598327637</v>
       </c>
       <c r="F5" t="n">
-        <v>21.21315956115723</v>
+        <v>21.12181282043457</v>
       </c>
     </row>
     <row r="6">
@@ -551,19 +551,19 @@
         <v>45839.16666666666</v>
       </c>
       <c r="B6" t="n">
-        <v>14.6568078994751</v>
+        <v>19.15325164794922</v>
       </c>
       <c r="C6" t="n">
-        <v>20.27652168273926</v>
+        <v>25.25820732116699</v>
       </c>
       <c r="D6" t="n">
-        <v>547.5282592773438</v>
+        <v>516.1005859375</v>
       </c>
       <c r="E6" t="n">
-        <v>15.34761810302734</v>
+        <v>17.11257743835449</v>
       </c>
       <c r="F6" t="n">
-        <v>20.0134105682373</v>
+        <v>18.54195976257324</v>
       </c>
     </row>
     <row r="7">
@@ -571,19 +571,19 @@
         <v>45839.20833333334</v>
       </c>
       <c r="B7" t="n">
-        <v>11.04688835144043</v>
+        <v>14.65497875213623</v>
       </c>
       <c r="C7" t="n">
-        <v>35.9573860168457</v>
+        <v>37.09440612792969</v>
       </c>
       <c r="D7" t="n">
-        <v>304.3837890625</v>
+        <v>351.1071472167969</v>
       </c>
       <c r="E7" t="n">
-        <v>10.94152545928955</v>
+        <v>13.44656276702881</v>
       </c>
       <c r="F7" t="n">
-        <v>30.37967872619629</v>
+        <v>22.62481689453125</v>
       </c>
     </row>
     <row r="8">
@@ -591,19 +591,19 @@
         <v>45839.25</v>
       </c>
       <c r="B8" t="n">
-        <v>15.04855346679688</v>
+        <v>16.8896484375</v>
       </c>
       <c r="C8" t="n">
-        <v>25.26027679443359</v>
+        <v>25.36528778076172</v>
       </c>
       <c r="D8" t="n">
-        <v>399.205078125</v>
+        <v>412.1278991699219</v>
       </c>
       <c r="E8" t="n">
-        <v>9.836292266845703</v>
+        <v>12.33457183837891</v>
       </c>
       <c r="F8" t="n">
-        <v>35.52939224243164</v>
+        <v>24.64070129394531</v>
       </c>
     </row>
     <row r="9">
@@ -611,19 +611,19 @@
         <v>45839.29166666666</v>
       </c>
       <c r="B9" t="n">
-        <v>14.98594570159912</v>
+        <v>15.65823364257812</v>
       </c>
       <c r="C9" t="n">
-        <v>31.84878921508789</v>
+        <v>31.56048202514648</v>
       </c>
       <c r="D9" t="n">
-        <v>394.1083984375</v>
+        <v>382.6197509765625</v>
       </c>
       <c r="E9" t="n">
-        <v>2.728171110153198</v>
+        <v>6.520807266235352</v>
       </c>
       <c r="F9" t="n">
-        <v>24.07693672180176</v>
+        <v>14.72403621673584</v>
       </c>
     </row>
     <row r="10">
@@ -631,19 +631,19 @@
         <v>45839.33333333334</v>
       </c>
       <c r="B10" t="n">
-        <v>11.12183380126953</v>
+        <v>12.05608654022217</v>
       </c>
       <c r="C10" t="n">
-        <v>21.38128280639648</v>
+        <v>19.16384696960449</v>
       </c>
       <c r="D10" t="n">
-        <v>359.3284912109375</v>
+        <v>356.1142883300781</v>
       </c>
       <c r="E10" t="n">
-        <v>7.637121200561523</v>
+        <v>9.992107391357422</v>
       </c>
       <c r="F10" t="n">
-        <v>23.30709075927734</v>
+        <v>13.52243328094482</v>
       </c>
     </row>
     <row r="11">
@@ -651,19 +651,19 @@
         <v>45839.375</v>
       </c>
       <c r="B11" t="n">
-        <v>13.85556316375732</v>
+        <v>12.86615085601807</v>
       </c>
       <c r="C11" t="n">
-        <v>28.51654624938965</v>
+        <v>26.69015693664551</v>
       </c>
       <c r="D11" t="n">
-        <v>358.5792846679688</v>
+        <v>344.4459228515625</v>
       </c>
       <c r="E11" t="n">
-        <v>6.047729969024658</v>
+        <v>6.602229595184326</v>
       </c>
       <c r="F11" t="n">
-        <v>28.98985862731934</v>
+        <v>16.96483421325684</v>
       </c>
     </row>
     <row r="12">
@@ -671,19 +671,19 @@
         <v>45839.41666666666</v>
       </c>
       <c r="B12" t="n">
-        <v>21.7485523223877</v>
+        <v>21.5193977355957</v>
       </c>
       <c r="C12" t="n">
-        <v>20.49127197265625</v>
+        <v>17.57468605041504</v>
       </c>
       <c r="D12" t="n">
-        <v>386.6887817382812</v>
+        <v>353.9507446289062</v>
       </c>
       <c r="E12" t="n">
-        <v>10.76991844177246</v>
+        <v>12.03373432159424</v>
       </c>
       <c r="F12" t="n">
-        <v>28.76893615722656</v>
+        <v>16.46114349365234</v>
       </c>
     </row>
     <row r="13">
@@ -691,19 +691,19 @@
         <v>45839.45833333334</v>
       </c>
       <c r="B13" t="n">
-        <v>18.42563438415527</v>
+        <v>16.37925910949707</v>
       </c>
       <c r="C13" t="n">
-        <v>26.61476707458496</v>
+        <v>21.54849815368652</v>
       </c>
       <c r="D13" t="n">
-        <v>407.2236633300781</v>
+        <v>430.1849365234375</v>
       </c>
       <c r="E13" t="n">
-        <v>7.482008457183838</v>
+        <v>8.580946922302246</v>
       </c>
       <c r="F13" t="n">
-        <v>19.90375137329102</v>
+        <v>10.13596248626709</v>
       </c>
     </row>
   </sheetData>

</xml_diff>